<commit_message>
Thêm chức năng quét ảnh bằng Claude Vision API và paste từ clipboard
- server.py: thêm endpoint POST /api/scan-images dùng Claude Vision (claude-opus-4-8) để OCR ảnh trong input/ và trả về JSON thông tin điền form
- index.html: thêm nút Quét thông tin bằng AI, hỗ trợ Ctrl+V dán ảnh từ clipboard vào upload zone
- requirements.txt: thêm anthropic>=0.40
- Xóa file docs/thong_tin_giam_dinh_xe_filled.xlsx không cần thiết

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/thong_tin_giam_dinh_xe.xlsx
+++ b/docs/thong_tin_giam_dinh_xe.xlsx
@@ -697,7 +697,11 @@
           <t>Giấy phép lưu hành</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>VA 3365650</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="8">
       <c r="A15" s="2" t="inlineStr">
@@ -1038,7 +1042,11 @@
           <t>Số hồ sơ</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="8">
       <c r="A38" s="2" t="inlineStr">
@@ -1051,7 +1059,11 @@
           <t>Mã giám định viên</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="8">
       <c r="A39" s="2" t="inlineStr">
@@ -1081,7 +1093,11 @@
           <t>Ngày giám định</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="8">
       <c r="A41" s="2" t="inlineStr">
@@ -1094,7 +1110,11 @@
           <t>Ngày vào gara</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22" customHeight="1" s="8">
       <c r="A42" s="7" t="inlineStr">
@@ -1131,7 +1151,11 @@
           <t>Giờ tai nạn</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1" s="8">
       <c r="A45" s="2" t="inlineStr">
@@ -1144,7 +1168,11 @@
           <t>Địa điểm tai nạn</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1" s="8">
       <c r="A46" s="2" t="inlineStr">
@@ -1157,7 +1185,11 @@
           <t>Diễn biến tai nạn</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1" s="8">
       <c r="A47" s="2" t="inlineStr">
@@ -1170,7 +1202,11 @@
           <t>Nguyên nhân</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1" s="8">
       <c r="A48" s="7" t="inlineStr">
@@ -1190,7 +1226,11 @@
           <t>Ngày hóa đơn</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="8">
       <c r="A50" s="2" t="inlineStr">
@@ -1203,7 +1243,11 @@
           <t>Tháng hóa đơn</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1" s="8">
       <c r="A51" s="2" t="inlineStr">
@@ -1216,7 +1260,11 @@
           <t>Năm hóa đơn</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="8">
       <c r="A52" s="2" t="inlineStr">
@@ -1229,7 +1277,11 @@
           <t>Tổng cộng tiền thanh toán</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr"/>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="22" customHeight="1" s="8">
       <c r="A53" s="7" t="inlineStr">
@@ -1249,7 +1301,11 @@
           <t>Tên gara</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr"/>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1" s="8">
       <c r="A55" s="2" t="inlineStr">
@@ -1262,7 +1318,11 @@
           <t>Số tài khoản</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1" s="8">
       <c r="A56" s="2" t="inlineStr">
@@ -1275,7 +1335,11 @@
           <t>Tên ngân hàng</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr"/>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1" s="8">
       <c r="A57" s="2" t="inlineStr">
@@ -1288,7 +1352,11 @@
           <t>Địa chỉ ngân hàng</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr"/>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="58"/>
     <row r="59">

</xml_diff>

<commit_message>
Sửa lỗi tên lái xe lấy nhầm chủ xe và tiền thanh toán bị rớt
1. Tên lái xe lấy nhầm sang chủ xe
   server.py tự copy chu_xe -> lai_xe (và dia_chi_chu_xe -> dia_chi_lai_xe)
   khi scan không ra lai_xe. Chủ xe thường là pháp nhân nên sinh ra tên lái
   xe sai, ví dụ "CÔNG TY TNHH PHÚC XUYÊN". Bỏ fallback này: không có nguồn
   thì để trống cho người dùng tự điền, đúng quy tắc "placeholder an toàn".
   Bổ sung SCAN_PROMPT cấm AI tự suy đoán lái xe từ chủ xe.

2. Số tiền thanh toán không ra số lẫn chữ
   Sheet "Thông tin" của docs/thong_tin_giam_dinh_xe.xlsx thiếu hẳn dòng
   {tien_tt} dù CLAUDE.md có ghi. save_excel() chỉ ghi key nào đã có dòng
   sẵn ở cột A nên tien_tt từ form bị rớt âm thầm, script đọc lại ra rỗng
   -> "Không đồng". Thêm dòng {tien_tt} vào nhóm G. TÀI CHÍNH.

Ghi chú CLAUDE.md: Excel là nút thắt dữ liệu (field mới phải thêm dòng vào
template), và insert_rows() của openpyxl không dịch merged range.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/thong_tin_giam_dinh_xe.xlsx
+++ b/docs/thong_tin_giam_dinh_xe.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" style="8" min="1" max="1"/>
@@ -1283,39 +1283,39 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1" s="8">
-      <c r="A53" s="7" t="inlineStr">
+    <row r="53" ht="18" customHeight="1" s="8">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>{tien_tt}</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Tiền thanh toán</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="8">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>H. GARA SỬA CHỮA</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1" s="8">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>{ten_gara}</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Tên gara</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>...</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1" s="8">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>{so_tk}</t>
+          <t>{ten_gara}</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Số tài khoản</t>
+          <t>Tên gara</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -1327,12 +1327,12 @@
     <row r="56" ht="18" customHeight="1" s="8">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>{ten_ngan_hang}</t>
+          <t>{so_tk}</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Tên ngân hàng</t>
+          <t>Số tài khoản</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -1344,23 +1344,40 @@
     <row r="57" ht="18" customHeight="1" s="8">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>{ten_ngan_hang}</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Tên ngân hàng</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>{dia_chi_ngan_hang}</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Địa chỉ ngân hàng</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>...</t>
         </is>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>💡 Chỉ điền vào cột C (Giá trị). Không thay đổi cột A và B.</t>
         </is>
@@ -1369,14 +1386,14 @@
   </sheetData>
   <autoFilter ref="A1:C57"/>
   <mergeCells count="8">
+    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A53:C53"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>